<commit_message>
changed LLM API setting in code
</commit_message>
<xml_diff>
--- a/Documents/AI Discovery Workshop/Nisol_Discovery_Assessment_Novatech_Simulation_LowMaturity.xlsx
+++ b/Documents/AI Discovery Workshop/Nisol_Discovery_Assessment_Novatech_Simulation_LowMaturity.xlsx
@@ -1364,12 +1364,12 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1997,13 +1997,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="32" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="33"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
+      <c r="A4" s="36" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="37"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
@@ -2066,16 +2066,16 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="32" t="s">
         <v>364</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="33" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="36"/>
-      <c r="B10" s="37"/>
+      <c r="A10" s="34"/>
+      <c r="B10" s="35"/>
     </row>
     <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">

</xml_diff>